<commit_message>
proj37: markdown popups (Markdig) + rename to Agentic Cost Estimation + Azure pricing references (UI+Excel) + non-prod/prod/total cost model (UI+Excel)
</commit_message>
<xml_diff>
--- a/proj37_foundry_cost_estimator_poc/samples/example-output-azure-cost-estimate.xlsx
+++ b/proj37_foundry_cost_estimator_poc/samples/example-output-azure-cost-estimate.xlsx
@@ -8,16 +8,22 @@
   <x:sheets>
     <x:sheet name="Summary" sheetId="1" r:id="rId2"/>
     <x:sheet name="Cost Model" sheetId="2" r:id="rId3"/>
-    <x:sheet name="Requirements" sheetId="3" r:id="rId4"/>
-    <x:sheet name="Scope" sheetId="4" r:id="rId5"/>
-    <x:sheet name="Documents" sheetId="5" r:id="rId6"/>
+    <x:sheet name="Non-Prod" sheetId="3" r:id="rId4"/>
+    <x:sheet name="Prod" sheetId="4" r:id="rId5"/>
+    <x:sheet name="Total" sheetId="5" r:id="rId6"/>
+    <x:sheet name="Requirements" sheetId="6" r:id="rId7"/>
+    <x:sheet name="Scope" sheetId="7" r:id="rId8"/>
+    <x:sheet name="Documents" sheetId="8" r:id="rId9"/>
   </x:sheets>
   <x:definedNames>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Requirements!$A$1:$E$13</x:definedName>
-    <x:definedName name="Proj37_MonthlySubtotal">'Cost Model'!$I$15:$I$15</x:definedName>
-    <x:definedName name="Proj37_Contingency">'Cost Model'!$B$17:$B$17</x:definedName>
-    <x:definedName name="Proj37_MonthlyTotal">'Cost Model'!$B$18:$B$18</x:definedName>
-    <x:definedName name="Proj37_AnnualTotal">'Cost Model'!$B$19:$B$19</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Requirements!$A$1:$E$13</x:definedName>
+    <x:definedName name="Proj37_MonthlySubtotal">'Cost Model'!$I$15</x:definedName>
+    <x:definedName name="Proj37_Contingency">'Cost Model'!$B$17</x:definedName>
+    <x:definedName name="Proj37_MonthlyTotal">'Cost Model'!$B$18</x:definedName>
+    <x:definedName name="Proj37_AnnualTotal">'Cost Model'!$B$19</x:definedName>
+    <x:definedName name="Proj37_NonProdMonthly">'Non-Prod'!$I$15</x:definedName>
+    <x:definedName name="Proj37_ProdMonthly">Prod!$I$15</x:definedName>
+    <x:definedName name="Proj37_TotalMonthly">Total!$J$15:$J$15</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="125725"/>
 </x:workbook>
@@ -35,13 +41,13 @@
     <x:t>Project</x:t>
   </x:si>
   <x:si>
-    <x:t>sample-statement-of-work.md</x:t>
+    <x:t>Contoso Document Intelligence Platform</x:t>
   </x:si>
   <x:si>
     <x:t>Job ID</x:t>
   </x:si>
   <x:si>
-    <x:t>48cd2c71d88f45ac980c532df35f9c76</x:t>
+    <x:t>68c7798ba5574490856d0426c99d4cc4</x:t>
   </x:si>
   <x:si>
     <x:t>Estimation engine</x:t>
@@ -110,6 +116,18 @@
     <x:t>Annual total (incl. contingency)</x:t>
   </x:si>
   <x:si>
+    <x:t>Cost by environment (monthly, incl. contingency)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Non-Prod monthly</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Prod monthly</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total monthly (Non-Prod + Prod)</x:t>
+  </x:si>
+  <x:si>
     <x:t>Disclaimer</x:t>
   </x:si>
   <x:si>
@@ -152,6 +170,9 @@
     <x:t>Monthly Cost</x:t>
   </x:si>
   <x:si>
+    <x:t>Pricing Reference</x:t>
+  </x:si>
+  <x:si>
     <x:t>AI</x:t>
   </x:si>
   <x:si>
@@ -170,6 +191,9 @@
     <x:t>per service/mo</x:t>
   </x:si>
   <x:si>
+    <x:t>Azure AI Search pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Microsoft Foundry (Azure OpenAI)</x:t>
   </x:si>
   <x:si>
@@ -185,6 +209,9 @@
     <x:t>per 1K tokens</x:t>
   </x:si>
   <x:si>
+    <x:t>Azure OpenAI pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>1K output tokens</x:t>
   </x:si>
   <x:si>
@@ -209,6 +236,9 @@
     <x:t>per instance/mo</x:t>
   </x:si>
   <x:si>
+    <x:t>App Service pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Azure Functions</x:t>
   </x:si>
   <x:si>
@@ -224,6 +254,9 @@
     <x:t>per 1M exec</x:t>
   </x:si>
   <x:si>
+    <x:t>Azure Functions pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Data</x:t>
   </x:si>
   <x:si>
@@ -242,6 +275,9 @@
     <x:t>per GB/mo</x:t>
   </x:si>
   <x:si>
+    <x:t>Blob Storage pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Azure SQL Database</x:t>
   </x:si>
   <x:si>
@@ -257,6 +293,9 @@
     <x:t>per vCore/mo</x:t>
   </x:si>
   <x:si>
+    <x:t>Azure SQL Database pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Networking</x:t>
   </x:si>
   <x:si>
@@ -275,6 +314,9 @@
     <x:t>per GB</x:t>
   </x:si>
   <x:si>
+    <x:t>Bandwidth pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Observability</x:t>
   </x:si>
   <x:si>
@@ -290,6 +332,9 @@
     <x:t>50 GB telemetry/mo</x:t>
   </x:si>
   <x:si>
+    <x:t>Azure Monitor pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Security</x:t>
   </x:si>
   <x:si>
@@ -305,6 +350,9 @@
     <x:t>per 10K ops</x:t>
   </x:si>
   <x:si>
+    <x:t>Key Vault pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t>Notes</x:t>
   </x:si>
   <x:si>
@@ -314,12 +362,57 @@
     <x:t>• Replace AzurePricingCatalog with the Azure Retail Prices API for production accuracy.</x:t>
   </x:si>
   <x:si>
+    <x:t>• Each line item links to its first-party Azure pricing page for audit (shown in UI and Excel).</x:t>
+  </x:si>
+  <x:si>
+    <x:t>• Non-prod view models a scaled-down dev/test footprint of the same architecture; Total = Non-prod + Prod.</x:t>
+  </x:si>
+  <x:si>
     <x:t>• Estimate scale assumptions: Large / enterprise (≈200k AI req/mo, multi-instance compute).</x:t>
   </x:si>
   <x:si>
     <x:t>• How to add a line item: select the last data row, press Tab/Enter to spill into the next row, then type your Category/Service plus a Quantity and Unit Price. Monthly Cost and the Monthly subtotal update automatically.</x:t>
   </x:si>
   <x:si>
+    <x:t>Non-Prod environment — monthly cost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scaled-down dev/test/POC footprint of the same architecture.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Prod environment — monthly cost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Full production sizing for the live workload.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total cost of ownership — Non-Prod + Prod</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Edit either quantity column; Non-Prod, Prod and Total costs recalculate automatically.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NonProd Qty</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Prod Qty</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NonProd Cost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Prod Cost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total Cost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total monthly (incl. contingency)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total annual (incl. contingency)</x:t>
+  </x:si>
+  <x:si>
     <x:t>ID</x:t>
   </x:si>
   <x:si>
@@ -539,10 +632,13 @@
     <x:t>Excerpt</x:t>
   </x:si>
   <x:si>
+    <x:t>01-contoso-document-intelligence-platform.md</x:t>
+  </x:si>
+  <x:si>
     <x:t>text/markdown</x:t>
   </x:si>
   <x:si>
-    <x:t># Project: Contoso Claims Intelligence Platform  ## Statement of Work (Technical Brief)  ### Business context Contoso Insurance receives thousands of claims documents (PDFs, scanned forms, emails) every day. The business wants an enterprise web application that lets claims handle…</x:t>
+    <x:t># Project: Contoso Document Intelligence Platform  ## Statement of Work (Technical Brief)  ### Business context Contoso Corporate Services receives thousands of inbound business documents (PDFs, scanned forms, emails) every day across procurement, HR, and facilities. The business…</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -556,7 +652,7 @@
     <x:numFmt numFmtId="166" formatCode="#,##0.######"/>
     <x:numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000000"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -601,6 +697,14 @@
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
       <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:u val="single"/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1A73E8"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
@@ -703,7 +807,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="19">
+  <x:cellStyleXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -746,6 +850,9 @@
     <x:xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="166" fontId="0" fillId="5" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -762,7 +869,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -828,6 +935,10 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -863,21 +974,27 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
   </x:cellStyles>
-  <x:dxfs count="1">
+  <x:dxfs count="2">
     <x:dxf>
       <x:font>
         <x:i/>
       </x:font>
       <x:numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:u val="single"/>
+        <x:color rgb="FF1A73E8"/>
+      </x:font>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CostModel" displayName="CostModel" ref="A4:I15" totalsRowCount="1">
-  <x:autoFilter ref="A4:I14"/>
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CostModel" displayName="CostModel" ref="A4:J15" totalsRowCount="1">
+  <x:autoFilter ref="A4:J14"/>
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="Category" totalsRowLabel="Monthly subtotal"/>
     <x:tableColumn id="2" name="Service"/>
     <x:tableColumn id="3" name="SKU / Tier"/>
@@ -889,8 +1006,77 @@
     <x:tableColumn id="9" name="Monthly Cost" totalsRowFunction="sum" dataDxfId="0">
       <x:calculatedColumnFormula>[@Quantity]*[@[Unit Price]]</x:calculatedColumnFormula>
     </x:tableColumn>
+    <x:tableColumn id="10" name="Pricing Reference" dataDxfId="1"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NonProdCost" displayName="NonProdCost" ref="A4:J15" totalsRowCount="1">
+  <x:autoFilter ref="A4:J14"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="Category" totalsRowLabel="Monthly subtotal"/>
+    <x:tableColumn id="2" name="Service"/>
+    <x:tableColumn id="3" name="SKU / Tier"/>
+    <x:tableColumn id="4" name="Meter"/>
+    <x:tableColumn id="5" name="Assumption"/>
+    <x:tableColumn id="6" name="Quantity"/>
+    <x:tableColumn id="7" name="Unit Price"/>
+    <x:tableColumn id="8" name="Unit"/>
+    <x:tableColumn id="9" name="Monthly Cost" totalsRowFunction="sum" dataDxfId="0">
+      <x:calculatedColumnFormula>[@Quantity]*[@[Unit Price]]</x:calculatedColumnFormula>
+    </x:tableColumn>
+    <x:tableColumn id="10" name="Pricing Reference" dataDxfId="1"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ProdCost" displayName="ProdCost" ref="A4:J15" totalsRowCount="1">
+  <x:autoFilter ref="A4:J14"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="Category" totalsRowLabel="Monthly subtotal"/>
+    <x:tableColumn id="2" name="Service"/>
+    <x:tableColumn id="3" name="SKU / Tier"/>
+    <x:tableColumn id="4" name="Meter"/>
+    <x:tableColumn id="5" name="Assumption"/>
+    <x:tableColumn id="6" name="Quantity"/>
+    <x:tableColumn id="7" name="Unit Price"/>
+    <x:tableColumn id="8" name="Unit"/>
+    <x:tableColumn id="9" name="Monthly Cost" totalsRowFunction="sum" dataDxfId="0">
+      <x:calculatedColumnFormula>[@Quantity]*[@[Unit Price]]</x:calculatedColumnFormula>
+    </x:tableColumn>
+    <x:tableColumn id="10" name="Pricing Reference" dataDxfId="1"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TotalCost" displayName="TotalCost" ref="A4:K15" totalsRowCount="1">
+  <x:autoFilter ref="A4:K14"/>
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Category" totalsRowLabel="Monthly subtotal"/>
+    <x:tableColumn id="2" name="Service"/>
+    <x:tableColumn id="3" name="SKU / Tier"/>
+    <x:tableColumn id="4" name="Unit Price"/>
+    <x:tableColumn id="5" name="Unit"/>
+    <x:tableColumn id="6" name="NonProd Qty"/>
+    <x:tableColumn id="7" name="Prod Qty"/>
+    <x:tableColumn id="8" name="NonProd Cost" totalsRowFunction="sum" dataDxfId="0">
+      <x:calculatedColumnFormula>[@[NonProd Qty]]*[@[Unit Price]]</x:calculatedColumnFormula>
+    </x:tableColumn>
+    <x:tableColumn id="9" name="Prod Cost" totalsRowFunction="sum" dataDxfId="0">
+      <x:calculatedColumnFormula>[@[Prod Qty]]*[@[Unit Price]]</x:calculatedColumnFormula>
+    </x:tableColumn>
+    <x:tableColumn id="10" name="Total Cost" totalsRowFunction="sum" dataDxfId="0">
+      <x:calculatedColumnFormula>[@[NonProd Cost]]+[@[Prod Cost]]</x:calculatedColumnFormula>
+    </x:tableColumn>
+    <x:tableColumn id="11" name="Pricing Reference" dataDxfId="1"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -1182,7 +1368,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:B24"/>
+  <x:dimension ref="A1:B29"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28.710625" style="0" customWidth="1"/>
@@ -1200,7 +1386,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="3">
-        <x:v>46187.3069106713</x:v>
+        <x:v>46194.0680423958</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:2">
@@ -1343,19 +1529,50 @@
       </x:c>
       <x:c r="B23" s="6"/>
     </x:row>
-    <x:row r="24" spans="1:2" ht="60" customHeight="1">
+    <x:row r="24" spans="1:2">
       <x:c r="A24" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B24" s="10" t="s">
+      <x:c r="B24" s="7">
+        <x:f>Proj37_NonProdMonthly*1.25</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:2">
+      <x:c r="A25" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="B25" s="7">
+        <x:f>Proj37_ProdMonthly*1.25</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:2">
+      <x:c r="A26" s="8" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B26" s="9">
+        <x:f>Proj37_TotalMonthly*1.25</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:2">
+      <x:c r="A28" s="5" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B28" s="6"/>
+    </x:row>
+    <x:row r="29" spans="1:2" ht="60" customHeight="1">
+      <x:c r="A29" s="4" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="s">
+        <x:v>34</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:mergeCells count="3">
+  <x:mergeCells count="4">
     <x:mergeCell ref="A1:B1"/>
     <x:mergeCell ref="A17:B17"/>
     <x:mergeCell ref="A23:B23"/>
+    <x:mergeCell ref="A28:B28"/>
   </x:mergeCells>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -1370,7 +1587,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I25"/>
+  <x:dimension ref="A1:J27"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
@@ -1381,11 +1598,12 @@
     <x:col min="6" max="6" width="12.710625" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="14.710625" style="0" customWidth="1"/>
     <x:col min="8" max="9" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:9" ht="26" customHeight="1">
+    <x:row r="1" spans="1:10" ht="26" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -1396,9 +1614,9 @@
       <x:c r="H1" s="2"/>
       <x:c r="I1" s="2"/>
     </x:row>
-    <x:row r="2" spans="1:9" ht="42" customHeight="1">
+    <x:row r="2" spans="1:10" ht="42" customHeight="1">
       <x:c r="A2" s="11" t="s">
-        <x:v>32</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -1409,50 +1627,53 @@
       <x:c r="H2" s="12"/>
       <x:c r="I2" s="12"/>
     </x:row>
-    <x:row r="4" spans="1:9">
+    <x:row r="4" spans="1:10">
       <x:c r="A4" s="13" t="s">
-        <x:v>33</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B4" s="13" t="s">
-        <x:v>34</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C4" s="13" t="s">
-        <x:v>35</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D4" s="13" t="s">
-        <x:v>36</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E4" s="13" t="s">
-        <x:v>37</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F4" s="13" t="s">
-        <x:v>38</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G4" s="13" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="H4" s="13" t="s">
-        <x:v>40</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="I4" s="13" t="s">
-        <x:v>41</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:9">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:10">
       <x:c r="A5" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="F5" s="14">
         <x:v>1</x:v>
@@ -1461,282 +1682,313 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="H5" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="I5" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="6" spans="1:9">
+      <x:c r="J5" s="17" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:10">
       <x:c r="A6" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F6" s="17">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F6" s="18">
         <x:v>800000</x:v>
       </x:c>
-      <x:c r="G6" s="18">
+      <x:c r="G6" s="19">
         <x:v>0.005</x:v>
       </x:c>
       <x:c r="H6" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="I6" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="7" spans="1:9">
+      <x:c r="J6" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:10">
       <x:c r="A7" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="F7" s="17">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F7" s="18">
         <x:v>240000</x:v>
       </x:c>
-      <x:c r="G7" s="18">
+      <x:c r="G7" s="19">
         <x:v>0.015</x:v>
       </x:c>
       <x:c r="H7" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="I7" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="8" spans="1:9">
+      <x:c r="J7" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:10">
       <x:c r="A8" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="F8" s="17">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F8" s="18">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G8" s="18">
+      <x:c r="G8" s="19">
         <x:v>259.88</x:v>
       </x:c>
       <x:c r="H8" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="I8" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="9" spans="1:9">
+      <x:c r="J8" s="17" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:10">
       <x:c r="A9" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F9" s="17">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="F9" s="18">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G9" s="18">
+      <x:c r="G9" s="19">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="H9" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="I9" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="10" spans="1:9">
+      <x:c r="J9" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:10">
       <x:c r="A10" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="F10" s="17">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="F10" s="18">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="G10" s="18">
+      <x:c r="G10" s="19">
         <x:v>0.021</x:v>
       </x:c>
       <x:c r="H10" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="I10" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="11" spans="1:9">
+      <x:c r="J10" s="17" t="s">
+        <x:v>81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:10">
       <x:c r="A11" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="F11" s="17">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F11" s="18">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G11" s="18">
+      <x:c r="G11" s="19">
         <x:v>130</x:v>
       </x:c>
       <x:c r="H11" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="I11" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="12" spans="1:9">
+      <x:c r="J11" s="17" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:10">
       <x:c r="A12" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="F12" s="17">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="F12" s="18">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="G12" s="18">
+      <x:c r="G12" s="19">
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="H12" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="I12" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="13" spans="1:9">
+      <x:c r="J12" s="17" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:10">
       <x:c r="A13" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="F13" s="17">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="F13" s="18">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="G13" s="18">
+      <x:c r="G13" s="19">
         <x:v>2.76</x:v>
       </x:c>
       <x:c r="H13" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="I13" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="14" spans="1:9">
+      <x:c r="J13" s="17" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:10">
       <x:c r="A14" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="F14" s="19">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="F14" s="20">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="G14" s="20">
+      <x:c r="G14" s="21">
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="H14" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="I14" s="16">
         <x:f>[@Quantity]*[@[Unit Price]]</x:f>
       </x:c>
-    </x:row>
-    <x:row r="15" spans="1:9">
+      <x:c r="J14" s="17" t="s">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:10">
       <x:c r="A15" s="4" t="s">
         <x:v>24</x:v>
       </x:c>
       <x:c r="I15" s="7">
         <x:f>SUBTOTAL(109,CostModel[Monthly Cost])</x:f>
       </x:c>
-    </x:row>
-    <x:row r="17" spans="1:9">
+      <x:c r="J15" s="17"/>
+    </x:row>
+    <x:row r="17" spans="1:10">
       <x:c r="A17" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
@@ -1744,7 +1996,7 @@
         <x:f>CostModel[[#Totals],[Monthly Cost]]*0.25</x:f>
       </x:c>
     </x:row>
-    <x:row r="18" spans="1:9">
+    <x:row r="18" spans="1:10">
       <x:c r="A18" s="8" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -1752,7 +2004,7 @@
         <x:f>CostModel[[#Totals],[Monthly Cost]]+B17</x:f>
       </x:c>
     </x:row>
-    <x:row r="19" spans="1:9">
+    <x:row r="19" spans="1:10">
       <x:c r="A19" s="8" t="s">
         <x:v>27</x:v>
       </x:c>
@@ -1760,29 +2012,39 @@
         <x:f>B18*12</x:f>
       </x:c>
     </x:row>
-    <x:row r="21" spans="1:9">
+    <x:row r="21" spans="1:10">
       <x:c r="A21" s="4" t="s">
-        <x:v>93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" spans="1:9">
+        <x:v>107</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:10">
       <x:c r="A22" s="0" t="s">
-        <x:v>94</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" spans="1:9">
+        <x:v>108</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:10">
       <x:c r="A23" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" spans="1:9">
+        <x:v>109</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:10">
       <x:c r="A24" s="0" t="s">
-        <x:v>96</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" spans="1:9">
-      <x:c r="A25" s="21" t="s">
-        <x:v>97</x:v>
+        <x:v>110</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:10">
+      <x:c r="A25" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:10">
+      <x:c r="A26" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:10">
+      <x:c r="A27" s="22" t="s">
+        <x:v>113</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1790,17 +2052,1412 @@
     <x:mergeCell ref="A1:I1"/>
     <x:mergeCell ref="A2:I2"/>
   </x:mergeCells>
+  <x:hyperlinks>
+    <x:hyperlink ref="J5" r:id="rId13"/>
+    <x:hyperlink ref="J6" r:id="rId14"/>
+    <x:hyperlink ref="J7" r:id="rId15"/>
+    <x:hyperlink ref="J8" r:id="rId16"/>
+    <x:hyperlink ref="J9" r:id="rId17"/>
+    <x:hyperlink ref="J10" r:id="rId18"/>
+    <x:hyperlink ref="J11" r:id="rId19"/>
+    <x:hyperlink ref="J12" r:id="rId20"/>
+    <x:hyperlink ref="J13" r:id="rId21"/>
+    <x:hyperlink ref="J14" r:id="rId22"/>
+  </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:tableParts count="1">
-    <x:tablePart r:id="rId9"/>
+    <x:tablePart r:id="rId12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:J19"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="45.710625" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.710625" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="8" max="9" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22.710625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:10" ht="26" customHeight="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+    </x:row>
+    <x:row r="2" spans="1:10">
+      <x:c r="A2" s="22" t="s">
+        <x:v>115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:10">
+      <x:c r="A4" s="13" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D4" s="13" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="G4" s="13" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:10">
+      <x:c r="A5" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="F5" s="14">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="G5" s="15">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I5" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J5" s="17" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:10">
+      <x:c r="A6" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F6" s="18">
+        <x:v>240000</x:v>
+      </x:c>
+      <x:c r="G6" s="19">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="I6" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J6" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:10">
+      <x:c r="A7" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F7" s="18">
+        <x:v>72000</x:v>
+      </x:c>
+      <x:c r="G7" s="19">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="I7" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J7" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:10">
+      <x:c r="A8" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F8" s="18">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="G8" s="19">
+        <x:v>259.88</x:v>
+      </x:c>
+      <x:c r="H8" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="I8" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J8" s="17" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:10">
+      <x:c r="A9" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="F9" s="18">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G9" s="19">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="I9" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J9" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:10">
+      <x:c r="A10" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="F10" s="18">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="G10" s="19">
+        <x:v>0.021</x:v>
+      </x:c>
+      <x:c r="H10" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="I10" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J10" s="17" t="s">
+        <x:v>81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:10">
+      <x:c r="A11" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F11" s="18">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="G11" s="19">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="H11" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="I11" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J11" s="17" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:10">
+      <x:c r="A12" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="F12" s="18">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="G12" s="19">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="H12" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="I12" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J12" s="17" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:10">
+      <x:c r="A13" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="E13" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="F13" s="18">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G13" s="19">
+        <x:v>2.76</x:v>
+      </x:c>
+      <x:c r="H13" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="I13" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J13" s="17" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:10">
+      <x:c r="A14" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="F14" s="20">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G14" s="21">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="H14" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="I14" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J14" s="17" t="s">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:10">
+      <x:c r="A15" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="I15" s="7">
+        <x:f>SUBTOTAL(109,NonProdCost[Monthly Cost])</x:f>
+      </x:c>
+      <x:c r="J15" s="17"/>
+    </x:row>
+    <x:row r="17" spans="1:10">
+      <x:c r="A17" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B17" s="7">
+        <x:f>NonProdCost[[#Totals],[Monthly Cost]]*0.25</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:10">
+      <x:c r="A18" s="8" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B18" s="9">
+        <x:f>NonProdCost[[#Totals],[Monthly Cost]]+B17</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:10">
+      <x:c r="A19" s="8" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B19" s="9">
+        <x:f>B18*12</x:f>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells count="1">
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:hyperlinks>
+    <x:hyperlink ref="J5" r:id="rId24"/>
+    <x:hyperlink ref="J6" r:id="rId25"/>
+    <x:hyperlink ref="J7" r:id="rId26"/>
+    <x:hyperlink ref="J8" r:id="rId27"/>
+    <x:hyperlink ref="J9" r:id="rId28"/>
+    <x:hyperlink ref="J10" r:id="rId29"/>
+    <x:hyperlink ref="J11" r:id="rId30"/>
+    <x:hyperlink ref="J12" r:id="rId31"/>
+    <x:hyperlink ref="J13" r:id="rId32"/>
+    <x:hyperlink ref="J14" r:id="rId33"/>
+  </x:hyperlinks>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="1">
+    <x:tablePart r:id="rId23"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:J19"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="45.710625" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.710625" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="8" max="9" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22.710625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:10" ht="26" customHeight="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+    </x:row>
+    <x:row r="2" spans="1:10">
+      <x:c r="A2" s="22" t="s">
+        <x:v>117</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:10">
+      <x:c r="A4" s="13" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D4" s="13" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="G4" s="13" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:10">
+      <x:c r="A5" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="F5" s="14">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="15">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="I5" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J5" s="17" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:10">
+      <x:c r="A6" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F6" s="18">
+        <x:v>800000</x:v>
+      </x:c>
+      <x:c r="G6" s="19">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="I6" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J6" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:10">
+      <x:c r="A7" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F7" s="18">
+        <x:v>240000</x:v>
+      </x:c>
+      <x:c r="G7" s="19">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="I7" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J7" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:10">
+      <x:c r="A8" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F8" s="18">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="19">
+        <x:v>259.88</x:v>
+      </x:c>
+      <x:c r="H8" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="I8" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J8" s="17" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:10">
+      <x:c r="A9" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="F9" s="18">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G9" s="19">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="I9" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J9" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:10">
+      <x:c r="A10" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="F10" s="18">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G10" s="19">
+        <x:v>0.021</x:v>
+      </x:c>
+      <x:c r="H10" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="I10" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J10" s="17" t="s">
+        <x:v>81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:10">
+      <x:c r="A11" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F11" s="18">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G11" s="19">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="H11" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="I11" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J11" s="17" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:10">
+      <x:c r="A12" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="F12" s="18">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G12" s="19">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="H12" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="I12" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J12" s="17" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:10">
+      <x:c r="A13" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="E13" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="F13" s="18">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G13" s="19">
+        <x:v>2.76</x:v>
+      </x:c>
+      <x:c r="H13" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="I13" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J13" s="17" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:10">
+      <x:c r="A14" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="F14" s="20">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="G14" s="21">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="H14" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="I14" s="16">
+        <x:f>[@Quantity]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J14" s="17" t="s">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:10">
+      <x:c r="A15" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="I15" s="7">
+        <x:f>SUBTOTAL(109,ProdCost[Monthly Cost])</x:f>
+      </x:c>
+      <x:c r="J15" s="17"/>
+    </x:row>
+    <x:row r="17" spans="1:10">
+      <x:c r="A17" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B17" s="7">
+        <x:f>ProdCost[[#Totals],[Monthly Cost]]*0.25</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:10">
+      <x:c r="A18" s="8" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B18" s="9">
+        <x:f>ProdCost[[#Totals],[Monthly Cost]]+B17</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:10">
+      <x:c r="A19" s="8" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B19" s="9">
+        <x:f>B18*12</x:f>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells count="1">
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:hyperlinks>
+    <x:hyperlink ref="J5" r:id="rId35"/>
+    <x:hyperlink ref="J6" r:id="rId36"/>
+    <x:hyperlink ref="J7" r:id="rId37"/>
+    <x:hyperlink ref="J8" r:id="rId38"/>
+    <x:hyperlink ref="J9" r:id="rId39"/>
+    <x:hyperlink ref="J10" r:id="rId40"/>
+    <x:hyperlink ref="J11" r:id="rId41"/>
+    <x:hyperlink ref="J12" r:id="rId42"/>
+    <x:hyperlink ref="J13" r:id="rId43"/>
+    <x:hyperlink ref="J14" r:id="rId44"/>
+  </x:hyperlinks>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="1">
+    <x:tablePart r:id="rId34"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:K19"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="5" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="6" max="7" width="12.710625" style="0" customWidth="1"/>
+    <x:col min="8" max="10" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22.710625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:11" ht="26" customHeight="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+    </x:row>
+    <x:row r="2" spans="1:11">
+      <x:c r="A2" s="22" t="s">
+        <x:v>119</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11">
+      <x:c r="A4" s="13" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D4" s="13" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G4" s="13" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="K4" s="13" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:11">
+      <x:c r="A5" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D5" s="15">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F5" s="14">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="G5" s="14">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I5" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J5" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K5" s="17" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:11">
+      <x:c r="A6" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D6" s="19">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="F6" s="18">
+        <x:v>240000</x:v>
+      </x:c>
+      <x:c r="G6" s="18">
+        <x:v>800000</x:v>
+      </x:c>
+      <x:c r="H6" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I6" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J6" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K6" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:11">
+      <x:c r="A7" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D7" s="19">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="F7" s="18">
+        <x:v>72000</x:v>
+      </x:c>
+      <x:c r="G7" s="18">
+        <x:v>240000</x:v>
+      </x:c>
+      <x:c r="H7" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I7" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J7" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K7" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:11">
+      <x:c r="A8" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D8" s="19">
+        <x:v>259.88</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F8" s="18">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="G8" s="18">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H8" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I8" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J8" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K8" s="17" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:11">
+      <x:c r="A9" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D9" s="19">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F9" s="18">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G9" s="18">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H9" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I9" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J9" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K9" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:11">
+      <x:c r="A10" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D10" s="19">
+        <x:v>0.021</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F10" s="18">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="G10" s="18">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="H10" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I10" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J10" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K10" s="17" t="s">
+        <x:v>81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:11">
+      <x:c r="A11" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D11" s="19">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="F11" s="18">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="G11" s="18">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H11" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I11" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J11" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K11" s="17" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:11">
+      <x:c r="A12" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D12" s="19">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F12" s="18">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="G12" s="18">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="H12" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I12" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J12" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K12" s="17" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:11">
+      <x:c r="A13" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D13" s="19">
+        <x:v>2.76</x:v>
+      </x:c>
+      <x:c r="E13" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F13" s="18">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G13" s="18">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H13" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I13" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J13" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K13" s="17" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:11">
+      <x:c r="A14" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D14" s="21">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="F14" s="20">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G14" s="20">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="H14" s="16">
+        <x:f>[@[NonProd Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="I14" s="16">
+        <x:f>[@[Prod Qty]]*[@[Unit Price]]</x:f>
+      </x:c>
+      <x:c r="J14" s="16">
+        <x:f>[@[NonProd Cost]]+[@[Prod Cost]]</x:f>
+      </x:c>
+      <x:c r="K14" s="17" t="s">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:11">
+      <x:c r="A15" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H15" s="7">
+        <x:f>SUBTOTAL(109,TotalCost[NonProd Cost])</x:f>
+      </x:c>
+      <x:c r="I15" s="7">
+        <x:f>SUBTOTAL(109,TotalCost[Prod Cost])</x:f>
+      </x:c>
+      <x:c r="J15" s="7">
+        <x:f>SUBTOTAL(109,TotalCost[Total Cost])</x:f>
+      </x:c>
+      <x:c r="K15" s="17"/>
+    </x:row>
+    <x:row r="17" spans="1:11">
+      <x:c r="A17" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B17" s="7">
+        <x:f>TotalCost[[#Totals],[Total Cost]]*0.25</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:11">
+      <x:c r="A18" s="8" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B18" s="9">
+        <x:f>TotalCost[[#Totals],[Total Cost]]+B17</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:11">
+      <x:c r="A19" s="8" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="B19" s="9">
+        <x:f>B18*12</x:f>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells count="1">
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:hyperlinks>
+    <x:hyperlink ref="K5" r:id="rId46"/>
+    <x:hyperlink ref="K6" r:id="rId47"/>
+    <x:hyperlink ref="K7" r:id="rId48"/>
+    <x:hyperlink ref="K8" r:id="rId49"/>
+    <x:hyperlink ref="K9" r:id="rId50"/>
+    <x:hyperlink ref="K10" r:id="rId51"/>
+    <x:hyperlink ref="K11" r:id="rId52"/>
+    <x:hyperlink ref="K12" r:id="rId53"/>
+    <x:hyperlink ref="K13" r:id="rId54"/>
+    <x:hyperlink ref="K14" r:id="rId55"/>
+  </x:hyperlinks>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="1">
+    <x:tablePart r:id="rId45"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1817,223 +3474,223 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="13" t="s">
-        <x:v>98</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B1" s="13" t="s">
-        <x:v>33</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C1" s="13" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="D1" s="22" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E1" s="22" t="s">
-        <x:v>101</x:v>
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D1" s="23" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E1" s="23" t="s">
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B2" s="12" t="s">
-        <x:v>55</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C2" s="12" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="D2" s="23" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="E2" s="23" t="s">
-        <x:v>105</x:v>
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D2" s="24" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="E2" s="24" t="s">
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D3" s="10" t="s">
-        <x:v>108</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="E3" s="10" t="s">
-        <x:v>109</x:v>
+        <x:v>138</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="12" t="s">
-        <x:v>110</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B4" s="12" t="s">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="12" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="D4" s="23" t="s">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="E4" s="23" t="s">
-        <x:v>112</x:v>
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D4" s="24" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="E4" s="24" t="s">
+        <x:v>141</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D5" s="10" t="s">
-        <x:v>114</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>115</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="12" t="s">
-        <x:v>116</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B6" s="12" t="s">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C6" s="12" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="D6" s="23" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="E6" s="23" t="s">
-        <x:v>118</x:v>
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D6" s="24" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="s">
+        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D7" s="10" t="s">
-        <x:v>120</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E7" s="10" t="s">
-        <x:v>121</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
       <x:c r="A8" s="12" t="s">
-        <x:v>122</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B8" s="12" t="s">
-        <x:v>55</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C8" s="12" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="D8" s="23" t="s">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="E8" s="23" t="s">
-        <x:v>125</x:v>
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="s">
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D9" s="10" t="s">
-        <x:v>127</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="E9" s="10" t="s">
-        <x:v>128</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:5">
       <x:c r="A10" s="12" t="s">
-        <x:v>129</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B10" s="12" t="s">
-        <x:v>88</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C10" s="12" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="D10" s="23" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="E10" s="23" t="s">
-        <x:v>131</x:v>
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="E10" s="24" t="s">
+        <x:v>160</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:5">
       <x:c r="A11" s="0" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>103</x:v>
-      </x:c>
       <x:c r="D11" s="10" t="s">
-        <x:v>133</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="E11" s="10" t="s">
-        <x:v>134</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:5">
       <x:c r="A12" s="12" t="s">
-        <x:v>135</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B12" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C12" s="12" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="D12" s="23" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="E12" s="23" t="s">
-        <x:v>137</x:v>
+      <x:c r="D12" s="24" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="E12" s="24" t="s">
+        <x:v>166</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:5">
       <x:c r="A13" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D13" s="10" t="s">
-        <x:v>139</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="E13" s="10" t="s">
-        <x:v>140</x:v>
+        <x:v>169</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2046,7 +3703,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2060,7 +3717,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:2" ht="26" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>141</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
     </x:row>
@@ -2074,18 +3731,18 @@
     </x:row>
     <x:row r="4" spans="1:2">
       <x:c r="A4" s="4" t="s">
-        <x:v>142</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B4" s="10" t="s">
-        <x:v>143</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:2">
       <x:c r="A5" s="4" t="s">
-        <x:v>144</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B5" s="10" t="s">
-        <x:v>145</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:2">
@@ -2122,91 +3779,91 @@
     </x:row>
     <x:row r="11" spans="1:2">
       <x:c r="A11" s="4" t="s">
-        <x:v>146</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:2">
       <x:c r="B12" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:2">
       <x:c r="B13" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:2">
       <x:c r="B14" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:2">
       <x:c r="B15" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:2">
       <x:c r="B16" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:2">
       <x:c r="B17" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:2">
       <x:c r="B18" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:2">
       <x:c r="B19" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:2">
       <x:c r="A21" s="4" t="s">
-        <x:v>156</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:2">
       <x:c r="B22" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:2">
       <x:c r="B23" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:2">
       <x:c r="A25" s="4" t="s">
-        <x:v>160</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:2">
       <x:c r="B26" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:2">
       <x:c r="B27" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:2">
       <x:c r="B28" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2221,7 +3878,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2229,7 +3886,7 @@
   <x:dimension ref="A1:F2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28.567768" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="43.853482" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="14.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="6.710625" style="0" customWidth="1"/>
@@ -2239,42 +3896,42 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="13" t="s">
-        <x:v>165</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B1" s="13" t="s">
-        <x:v>166</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="C1" s="13" t="s">
-        <x:v>167</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="D1" s="13" t="s">
-        <x:v>168</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E1" s="13" t="s">
-        <x:v>169</x:v>
-      </x:c>
-      <x:c r="F1" s="22" t="s">
-        <x:v>170</x:v>
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="F1" s="23" t="s">
+        <x:v>199</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
       <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>2431</x:v>
+        <x:v>2503</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>348</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>2431</x:v>
+        <x:v>2503</x:v>
       </x:c>
       <x:c r="F2" s="10" t="s">
-        <x:v>172</x:v>
+        <x:v>202</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
proj37: fix xlsx open-integrity + formula recalc (calcPr calcId=0/fullCalcOnLoad/forceFullCalc, drop stale calcChain.xml)
</commit_message>
<xml_diff>
--- a/proj37_foundry_cost_estimator_poc/samples/example-output-azure-cost-estimate.xlsx
+++ b/proj37_foundry_cost_estimator_poc/samples/example-output-azure-cost-estimate.xlsx
@@ -25,7 +25,7 @@
     <x:definedName name="Proj37_ProdMonthly">Prod!$I$15</x:definedName>
     <x:definedName name="Proj37_TotalMonthly">Total!$J$15:$J$15</x:definedName>
   </x:definedNames>
-  <x:calcPr calcId="125725"/>
+  <x:calcPr calcId="0" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </x:workbook>
 </file>
 
@@ -41,13 +41,13 @@
     <x:t>Project</x:t>
   </x:si>
   <x:si>
-    <x:t>Contoso Document Intelligence Platform</x:t>
+    <x:t>01-contoso-document-intelligence-platform</x:t>
   </x:si>
   <x:si>
     <x:t>Job ID</x:t>
   </x:si>
   <x:si>
-    <x:t>68c7798ba5574490856d0426c99d4cc4</x:t>
+    <x:t>d49a2e3fac054fd7846f56f30dd245b0</x:t>
   </x:si>
   <x:si>
     <x:t>Estimation engine</x:t>
@@ -77,7 +77,7 @@
     <x:t>Environment</x:t>
   </x:si>
   <x:si>
-    <x:t>non-production (POC/dev)</x:t>
+    <x:t>production</x:t>
   </x:si>
   <x:si>
     <x:t>Region</x:t>
@@ -197,7 +197,7 @@
     <x:t>Microsoft Foundry (Azure OpenAI)</x:t>
   </x:si>
   <x:si>
-    <x:t>gpt-5.4</x:t>
+    <x:t>gpt-4o</x:t>
   </x:si>
   <x:si>
     <x:t>1K input tokens</x:t>
@@ -452,7 +452,7 @@
     <x:t>REQ-003</x:t>
   </x:si>
   <x:si>
-    <x:t>Use a Microsoft Foundry prompt agent on model deployment 'gpt-5.4' for document understanding and estimation reasoning.</x:t>
+    <x:t>Use a Microsoft Foundry prompt agent on model deployment 'gpt-4o' for document understanding and estimation reasoning.</x:t>
   </x:si>
   <x:si>
     <x:t>Centralised, governed model access with content safety and identity.</x:t>
@@ -635,10 +635,10 @@
     <x:t>01-contoso-document-intelligence-platform.md</x:t>
   </x:si>
   <x:si>
-    <x:t>text/markdown</x:t>
-  </x:si>
-  <x:si>
-    <x:t># Project: Contoso Document Intelligence Platform  ## Statement of Work (Technical Brief)  ### Business context Contoso Corporate Services receives thousands of inbound business documents (PDFs, scanned forms, emails) every day across procurement, HR, and facilities. The business…</x:t>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>Enterprise document intelligence platform...</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1386,7 +1386,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="3">
-        <x:v>46194.0680423958</x:v>
+        <x:v>46196.1911887384</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:2">
@@ -3887,11 +3887,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="43.853482" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="6.710625" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.424911" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="80.710625" style="10" customWidth="1"/>
+    <x:col min="6" max="6" width="40.710625" style="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6">
@@ -3922,13 +3922,13 @@
         <x:v>201</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>2503</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>355</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>2503</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F2" s="10" t="s">
         <x:v>202</x:v>

</xml_diff>